<commit_message>
PAFS: Fixing the funding source defects
</commit_message>
<xml_diff>
--- a/src/plugins/downloads/helpers/fcerm1/fcerm1_template.xlsx
+++ b/src/plugins/downloads/helpers/fcerm1/fcerm1_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/795110/Documents/Fujale-Space/Work/Projects/EA/FCRM/PAFs/Remote/migration/pafs-backend-api/src/plugins/downloads/helpers/fcerm1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF37731B-D2B5-9F44-A18A-33B688FC8F50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED701F2F-7F91-5245-B119-531D733FD5E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-2800" yWindow="-21000" windowWidth="38400" windowHeight="21000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master local choices'!$A$6:$MZ$6</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1332,7 +1332,7 @@
     <t>PSO Name</t>
   </si>
   <si>
-    <t>PAFS Base 2026/27</t>
+    <t>PAFS Base 2023/24</t>
   </si>
 </sst>
 </file>
@@ -1862,101 +1862,101 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="11" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="17" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="21" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="22" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="20" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="16" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="17" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="18" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="11" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="10">
@@ -2269,10 +2269,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:374" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="73"/>
+      <c r="B1" s="62"/>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
       <c r="E1" s="8"/>
@@ -2647,10 +2647,10 @@
       <c r="NJ1" s="15"/>
     </row>
     <row r="2" spans="1:374" ht="28.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="74" t="s">
+      <c r="A2" s="63" t="s">
         <v>421</v>
       </c>
-      <c r="B2" s="74"/>
+      <c r="B2" s="63"/>
       <c r="C2" s="7"/>
       <c r="D2" s="16"/>
       <c r="E2" s="8"/>
@@ -3401,530 +3401,530 @@
       <c r="NJ3" s="15"/>
     </row>
     <row r="4" spans="1:374" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="75" t="s">
+      <c r="A4" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="76" t="s">
+      <c r="B4" s="64"/>
+      <c r="C4" s="65" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="76"/>
-      <c r="E4" s="76"/>
-      <c r="F4" s="76"/>
-      <c r="G4" s="76"/>
-      <c r="H4" s="76"/>
-      <c r="I4" s="77" t="s">
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="65"/>
+      <c r="H4" s="65"/>
+      <c r="I4" s="66" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="77"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="77"/>
-      <c r="M4" s="77"/>
-      <c r="N4" s="68" t="s">
+      <c r="J4" s="66"/>
+      <c r="K4" s="66"/>
+      <c r="L4" s="66"/>
+      <c r="M4" s="66"/>
+      <c r="N4" s="67" t="s">
         <v>4</v>
       </c>
-      <c r="O4" s="68"/>
-      <c r="P4" s="68"/>
-      <c r="Q4" s="69" t="s">
+      <c r="O4" s="67"/>
+      <c r="P4" s="67"/>
+      <c r="Q4" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="R4" s="69"/>
-      <c r="S4" s="69"/>
-      <c r="T4" s="69"/>
-      <c r="U4" s="69"/>
-      <c r="V4" s="70" t="s">
+      <c r="R4" s="68"/>
+      <c r="S4" s="68"/>
+      <c r="T4" s="68"/>
+      <c r="U4" s="68"/>
+      <c r="V4" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="W4" s="70"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="70"/>
-      <c r="Z4" s="70"/>
-      <c r="AA4" s="70"/>
-      <c r="AB4" s="70"/>
-      <c r="AC4" s="71" t="s">
+      <c r="W4" s="69"/>
+      <c r="X4" s="69"/>
+      <c r="Y4" s="69"/>
+      <c r="Z4" s="69"/>
+      <c r="AA4" s="69"/>
+      <c r="AB4" s="69"/>
+      <c r="AC4" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="AD4" s="71"/>
-      <c r="AE4" s="71"/>
-      <c r="AF4" s="72" t="s">
+      <c r="AD4" s="70"/>
+      <c r="AE4" s="70"/>
+      <c r="AF4" s="71" t="s">
         <v>8</v>
       </c>
-      <c r="AG4" s="72"/>
-      <c r="AH4" s="66"/>
-      <c r="AI4" s="66"/>
-      <c r="AJ4" s="66"/>
-      <c r="AK4" s="66"/>
-      <c r="AL4" s="66"/>
-      <c r="AM4" s="67" t="s">
+      <c r="AG4" s="71"/>
+      <c r="AH4" s="72"/>
+      <c r="AI4" s="72"/>
+      <c r="AJ4" s="72"/>
+      <c r="AK4" s="72"/>
+      <c r="AL4" s="72"/>
+      <c r="AM4" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="AN4" s="67"/>
-      <c r="AO4" s="67"/>
-      <c r="AP4" s="67"/>
-      <c r="AQ4" s="67"/>
-      <c r="AR4" s="67"/>
-      <c r="AS4" s="67"/>
-      <c r="AT4" s="67"/>
-      <c r="AU4" s="67"/>
-      <c r="AV4" s="67"/>
-      <c r="AW4" s="67"/>
-      <c r="AX4" s="67"/>
-      <c r="AY4" s="67"/>
-      <c r="AZ4" s="67"/>
-      <c r="BA4" s="67"/>
-      <c r="BB4" s="67"/>
-      <c r="BC4" s="67"/>
-      <c r="BD4" s="67"/>
-      <c r="BE4" s="67"/>
-      <c r="BF4" s="67"/>
-      <c r="BG4" s="67"/>
-      <c r="BH4" s="67"/>
-      <c r="BI4" s="67"/>
-      <c r="BJ4" s="67"/>
-      <c r="BK4" s="67"/>
-      <c r="BL4" s="67"/>
-      <c r="BM4" s="67"/>
-      <c r="BN4" s="67"/>
-      <c r="BO4" s="56" t="s">
+      <c r="AN4" s="73"/>
+      <c r="AO4" s="73"/>
+      <c r="AP4" s="73"/>
+      <c r="AQ4" s="73"/>
+      <c r="AR4" s="73"/>
+      <c r="AS4" s="73"/>
+      <c r="AT4" s="73"/>
+      <c r="AU4" s="73"/>
+      <c r="AV4" s="73"/>
+      <c r="AW4" s="73"/>
+      <c r="AX4" s="73"/>
+      <c r="AY4" s="73"/>
+      <c r="AZ4" s="73"/>
+      <c r="BA4" s="73"/>
+      <c r="BB4" s="73"/>
+      <c r="BC4" s="73"/>
+      <c r="BD4" s="73"/>
+      <c r="BE4" s="73"/>
+      <c r="BF4" s="73"/>
+      <c r="BG4" s="73"/>
+      <c r="BH4" s="73"/>
+      <c r="BI4" s="73"/>
+      <c r="BJ4" s="73"/>
+      <c r="BK4" s="73"/>
+      <c r="BL4" s="73"/>
+      <c r="BM4" s="73"/>
+      <c r="BN4" s="73"/>
+      <c r="BO4" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="BP4" s="56"/>
-      <c r="BQ4" s="56"/>
-      <c r="BR4" s="56"/>
-      <c r="BS4" s="56"/>
-      <c r="BT4" s="56"/>
-      <c r="BU4" s="56"/>
-      <c r="BV4" s="56"/>
-      <c r="BW4" s="56"/>
-      <c r="BX4" s="56"/>
-      <c r="BY4" s="65" t="s">
+      <c r="BP4" s="74"/>
+      <c r="BQ4" s="74"/>
+      <c r="BR4" s="74"/>
+      <c r="BS4" s="74"/>
+      <c r="BT4" s="74"/>
+      <c r="BU4" s="74"/>
+      <c r="BV4" s="74"/>
+      <c r="BW4" s="74"/>
+      <c r="BX4" s="74"/>
+      <c r="BY4" s="75" t="s">
         <v>11</v>
       </c>
-      <c r="BZ4" s="65"/>
-      <c r="CA4" s="65"/>
-      <c r="CB4" s="65"/>
-      <c r="CC4" s="65"/>
-      <c r="CD4" s="65"/>
-      <c r="CE4" s="65"/>
-      <c r="CF4" s="65"/>
-      <c r="CG4" s="65"/>
-      <c r="CH4" s="65"/>
-      <c r="CI4" s="60" t="s">
+      <c r="BZ4" s="75"/>
+      <c r="CA4" s="75"/>
+      <c r="CB4" s="75"/>
+      <c r="CC4" s="75"/>
+      <c r="CD4" s="75"/>
+      <c r="CE4" s="75"/>
+      <c r="CF4" s="75"/>
+      <c r="CG4" s="75"/>
+      <c r="CH4" s="75"/>
+      <c r="CI4" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="CJ4" s="60"/>
-      <c r="CK4" s="60"/>
-      <c r="CL4" s="60"/>
-      <c r="CM4" s="60"/>
-      <c r="CN4" s="60"/>
-      <c r="CO4" s="60"/>
-      <c r="CP4" s="60"/>
-      <c r="CQ4" s="60"/>
-      <c r="CR4" s="60"/>
-      <c r="CS4" s="65" t="s">
+      <c r="CJ4" s="76"/>
+      <c r="CK4" s="76"/>
+      <c r="CL4" s="76"/>
+      <c r="CM4" s="76"/>
+      <c r="CN4" s="76"/>
+      <c r="CO4" s="76"/>
+      <c r="CP4" s="76"/>
+      <c r="CQ4" s="76"/>
+      <c r="CR4" s="76"/>
+      <c r="CS4" s="75" t="s">
         <v>13</v>
       </c>
-      <c r="CT4" s="65"/>
-      <c r="CU4" s="65"/>
-      <c r="CV4" s="65"/>
-      <c r="CW4" s="65"/>
-      <c r="CX4" s="65"/>
-      <c r="CY4" s="65"/>
-      <c r="CZ4" s="65"/>
-      <c r="DA4" s="65"/>
-      <c r="DB4" s="65"/>
-      <c r="DC4" s="60" t="s">
+      <c r="CT4" s="75"/>
+      <c r="CU4" s="75"/>
+      <c r="CV4" s="75"/>
+      <c r="CW4" s="75"/>
+      <c r="CX4" s="75"/>
+      <c r="CY4" s="75"/>
+      <c r="CZ4" s="75"/>
+      <c r="DA4" s="75"/>
+      <c r="DB4" s="75"/>
+      <c r="DC4" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="DD4" s="60"/>
-      <c r="DE4" s="60"/>
-      <c r="DF4" s="60"/>
-      <c r="DG4" s="60"/>
-      <c r="DH4" s="60"/>
-      <c r="DI4" s="60"/>
-      <c r="DJ4" s="60"/>
-      <c r="DK4" s="60"/>
-      <c r="DL4" s="60"/>
-      <c r="DM4" s="65" t="s">
+      <c r="DD4" s="76"/>
+      <c r="DE4" s="76"/>
+      <c r="DF4" s="76"/>
+      <c r="DG4" s="76"/>
+      <c r="DH4" s="76"/>
+      <c r="DI4" s="76"/>
+      <c r="DJ4" s="76"/>
+      <c r="DK4" s="76"/>
+      <c r="DL4" s="76"/>
+      <c r="DM4" s="75" t="s">
         <v>15</v>
       </c>
-      <c r="DN4" s="65"/>
-      <c r="DO4" s="65"/>
-      <c r="DP4" s="65"/>
-      <c r="DQ4" s="65"/>
-      <c r="DR4" s="65"/>
-      <c r="DS4" s="65"/>
-      <c r="DT4" s="65"/>
-      <c r="DU4" s="65"/>
-      <c r="DV4" s="65"/>
-      <c r="DW4" s="60" t="s">
+      <c r="DN4" s="75"/>
+      <c r="DO4" s="75"/>
+      <c r="DP4" s="75"/>
+      <c r="DQ4" s="75"/>
+      <c r="DR4" s="75"/>
+      <c r="DS4" s="75"/>
+      <c r="DT4" s="75"/>
+      <c r="DU4" s="75"/>
+      <c r="DV4" s="75"/>
+      <c r="DW4" s="76" t="s">
         <v>16</v>
       </c>
-      <c r="DX4" s="60"/>
-      <c r="DY4" s="60"/>
-      <c r="DZ4" s="60"/>
-      <c r="EA4" s="60"/>
-      <c r="EB4" s="60"/>
-      <c r="EC4" s="60"/>
-      <c r="ED4" s="60"/>
-      <c r="EE4" s="60"/>
-      <c r="EF4" s="60"/>
-      <c r="EG4" s="65" t="s">
+      <c r="DX4" s="76"/>
+      <c r="DY4" s="76"/>
+      <c r="DZ4" s="76"/>
+      <c r="EA4" s="76"/>
+      <c r="EB4" s="76"/>
+      <c r="EC4" s="76"/>
+      <c r="ED4" s="76"/>
+      <c r="EE4" s="76"/>
+      <c r="EF4" s="76"/>
+      <c r="EG4" s="75" t="s">
         <v>17</v>
       </c>
-      <c r="EH4" s="65"/>
-      <c r="EI4" s="65"/>
-      <c r="EJ4" s="65"/>
-      <c r="EK4" s="65"/>
-      <c r="EL4" s="65"/>
-      <c r="EM4" s="65"/>
-      <c r="EN4" s="65"/>
-      <c r="EO4" s="65"/>
-      <c r="EP4" s="65"/>
-      <c r="EQ4" s="60" t="s">
+      <c r="EH4" s="75"/>
+      <c r="EI4" s="75"/>
+      <c r="EJ4" s="75"/>
+      <c r="EK4" s="75"/>
+      <c r="EL4" s="75"/>
+      <c r="EM4" s="75"/>
+      <c r="EN4" s="75"/>
+      <c r="EO4" s="75"/>
+      <c r="EP4" s="75"/>
+      <c r="EQ4" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="ER4" s="60"/>
-      <c r="ES4" s="60"/>
-      <c r="ET4" s="60"/>
-      <c r="EU4" s="60"/>
-      <c r="EV4" s="60"/>
-      <c r="EW4" s="60"/>
-      <c r="EX4" s="60"/>
-      <c r="EY4" s="60"/>
-      <c r="EZ4" s="60"/>
-      <c r="FA4" s="61" t="s">
+      <c r="ER4" s="76"/>
+      <c r="ES4" s="76"/>
+      <c r="ET4" s="76"/>
+      <c r="EU4" s="76"/>
+      <c r="EV4" s="76"/>
+      <c r="EW4" s="76"/>
+      <c r="EX4" s="76"/>
+      <c r="EY4" s="76"/>
+      <c r="EZ4" s="76"/>
+      <c r="FA4" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="FB4" s="61"/>
-      <c r="FC4" s="61"/>
-      <c r="FD4" s="61"/>
-      <c r="FE4" s="61"/>
-      <c r="FF4" s="61"/>
-      <c r="FG4" s="61"/>
-      <c r="FH4" s="61"/>
-      <c r="FI4" s="61"/>
-      <c r="FJ4" s="61"/>
-      <c r="FK4" s="62" t="s">
+      <c r="FB4" s="77"/>
+      <c r="FC4" s="77"/>
+      <c r="FD4" s="77"/>
+      <c r="FE4" s="77"/>
+      <c r="FF4" s="77"/>
+      <c r="FG4" s="77"/>
+      <c r="FH4" s="77"/>
+      <c r="FI4" s="77"/>
+      <c r="FJ4" s="77"/>
+      <c r="FK4" s="78" t="s">
         <v>20</v>
       </c>
-      <c r="FL4" s="62"/>
-      <c r="FM4" s="62"/>
-      <c r="FN4" s="62"/>
-      <c r="FO4" s="62"/>
-      <c r="FP4" s="62"/>
-      <c r="FQ4" s="62"/>
-      <c r="FR4" s="62"/>
-      <c r="FS4" s="62"/>
-      <c r="FT4" s="62"/>
-      <c r="FU4" s="63" t="s">
+      <c r="FL4" s="78"/>
+      <c r="FM4" s="78"/>
+      <c r="FN4" s="78"/>
+      <c r="FO4" s="78"/>
+      <c r="FP4" s="78"/>
+      <c r="FQ4" s="78"/>
+      <c r="FR4" s="78"/>
+      <c r="FS4" s="78"/>
+      <c r="FT4" s="78"/>
+      <c r="FU4" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="FV4" s="63"/>
-      <c r="FW4" s="63"/>
-      <c r="FX4" s="63"/>
-      <c r="FY4" s="63"/>
-      <c r="FZ4" s="63"/>
-      <c r="GA4" s="63"/>
-      <c r="GB4" s="63"/>
-      <c r="GC4" s="63"/>
-      <c r="GD4" s="63"/>
-      <c r="GE4" s="64" t="s">
+      <c r="FV4" s="79"/>
+      <c r="FW4" s="79"/>
+      <c r="FX4" s="79"/>
+      <c r="FY4" s="79"/>
+      <c r="FZ4" s="79"/>
+      <c r="GA4" s="79"/>
+      <c r="GB4" s="79"/>
+      <c r="GC4" s="79"/>
+      <c r="GD4" s="79"/>
+      <c r="GE4" s="80" t="s">
         <v>22</v>
       </c>
-      <c r="GF4" s="64"/>
-      <c r="GG4" s="64"/>
-      <c r="GH4" s="64"/>
-      <c r="GI4" s="64"/>
-      <c r="GJ4" s="64"/>
-      <c r="GK4" s="64"/>
-      <c r="GL4" s="64"/>
-      <c r="GM4" s="64"/>
-      <c r="GN4" s="64"/>
-      <c r="GO4" s="58" t="s">
+      <c r="GF4" s="80"/>
+      <c r="GG4" s="80"/>
+      <c r="GH4" s="80"/>
+      <c r="GI4" s="80"/>
+      <c r="GJ4" s="80"/>
+      <c r="GK4" s="80"/>
+      <c r="GL4" s="80"/>
+      <c r="GM4" s="80"/>
+      <c r="GN4" s="80"/>
+      <c r="GO4" s="81" t="s">
         <v>23</v>
       </c>
-      <c r="GP4" s="58"/>
-      <c r="GQ4" s="58"/>
-      <c r="GR4" s="58"/>
-      <c r="GS4" s="58"/>
-      <c r="GT4" s="58"/>
-      <c r="GU4" s="58"/>
-      <c r="GV4" s="58"/>
-      <c r="GW4" s="58"/>
-      <c r="GX4" s="58"/>
-      <c r="GY4" s="59" t="s">
+      <c r="GP4" s="81"/>
+      <c r="GQ4" s="81"/>
+      <c r="GR4" s="81"/>
+      <c r="GS4" s="81"/>
+      <c r="GT4" s="81"/>
+      <c r="GU4" s="81"/>
+      <c r="GV4" s="81"/>
+      <c r="GW4" s="81"/>
+      <c r="GX4" s="81"/>
+      <c r="GY4" s="82" t="s">
         <v>24</v>
       </c>
-      <c r="GZ4" s="59"/>
-      <c r="HA4" s="59"/>
-      <c r="HB4" s="59"/>
-      <c r="HC4" s="59"/>
-      <c r="HD4" s="59"/>
-      <c r="HE4" s="59"/>
-      <c r="HF4" s="59"/>
-      <c r="HG4" s="59"/>
-      <c r="HH4" s="59"/>
-      <c r="HI4" s="56" t="s">
+      <c r="GZ4" s="82"/>
+      <c r="HA4" s="82"/>
+      <c r="HB4" s="82"/>
+      <c r="HC4" s="82"/>
+      <c r="HD4" s="82"/>
+      <c r="HE4" s="82"/>
+      <c r="HF4" s="82"/>
+      <c r="HG4" s="82"/>
+      <c r="HH4" s="82"/>
+      <c r="HI4" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="HJ4" s="56"/>
-      <c r="HK4" s="56"/>
-      <c r="HL4" s="56"/>
-      <c r="HM4" s="56"/>
-      <c r="HN4" s="56"/>
-      <c r="HO4" s="56"/>
-      <c r="HP4" s="56"/>
-      <c r="HQ4" s="56"/>
-      <c r="HR4" s="56"/>
-      <c r="HS4" s="56" t="s">
+      <c r="HJ4" s="74"/>
+      <c r="HK4" s="74"/>
+      <c r="HL4" s="74"/>
+      <c r="HM4" s="74"/>
+      <c r="HN4" s="74"/>
+      <c r="HO4" s="74"/>
+      <c r="HP4" s="74"/>
+      <c r="HQ4" s="74"/>
+      <c r="HR4" s="74"/>
+      <c r="HS4" s="74" t="s">
         <v>26</v>
       </c>
-      <c r="HT4" s="56"/>
-      <c r="HU4" s="56"/>
-      <c r="HV4" s="56"/>
-      <c r="HW4" s="56"/>
-      <c r="HX4" s="56"/>
-      <c r="HY4" s="56"/>
-      <c r="HZ4" s="56"/>
-      <c r="IA4" s="56"/>
-      <c r="IB4" s="56"/>
-      <c r="IC4" s="56" t="s">
+      <c r="HT4" s="74"/>
+      <c r="HU4" s="74"/>
+      <c r="HV4" s="74"/>
+      <c r="HW4" s="74"/>
+      <c r="HX4" s="74"/>
+      <c r="HY4" s="74"/>
+      <c r="HZ4" s="74"/>
+      <c r="IA4" s="74"/>
+      <c r="IB4" s="74"/>
+      <c r="IC4" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="ID4" s="56"/>
-      <c r="IE4" s="56"/>
-      <c r="IF4" s="56"/>
-      <c r="IG4" s="56"/>
-      <c r="IH4" s="56"/>
-      <c r="II4" s="56"/>
-      <c r="IJ4" s="56"/>
-      <c r="IK4" s="56"/>
-      <c r="IL4" s="56"/>
-      <c r="IM4" s="56" t="s">
+      <c r="ID4" s="74"/>
+      <c r="IE4" s="74"/>
+      <c r="IF4" s="74"/>
+      <c r="IG4" s="74"/>
+      <c r="IH4" s="74"/>
+      <c r="II4" s="74"/>
+      <c r="IJ4" s="74"/>
+      <c r="IK4" s="74"/>
+      <c r="IL4" s="74"/>
+      <c r="IM4" s="74" t="s">
         <v>28</v>
       </c>
-      <c r="IN4" s="56"/>
-      <c r="IO4" s="56"/>
-      <c r="IP4" s="56"/>
-      <c r="IQ4" s="56"/>
-      <c r="IR4" s="56"/>
-      <c r="IS4" s="56"/>
-      <c r="IT4" s="56"/>
-      <c r="IU4" s="56"/>
-      <c r="IV4" s="56"/>
-      <c r="IW4" s="56" t="s">
+      <c r="IN4" s="74"/>
+      <c r="IO4" s="74"/>
+      <c r="IP4" s="74"/>
+      <c r="IQ4" s="74"/>
+      <c r="IR4" s="74"/>
+      <c r="IS4" s="74"/>
+      <c r="IT4" s="74"/>
+      <c r="IU4" s="74"/>
+      <c r="IV4" s="74"/>
+      <c r="IW4" s="74" t="s">
         <v>29</v>
       </c>
-      <c r="IX4" s="56"/>
-      <c r="IY4" s="56"/>
-      <c r="IZ4" s="56"/>
-      <c r="JA4" s="56"/>
-      <c r="JB4" s="56"/>
-      <c r="JC4" s="56"/>
-      <c r="JD4" s="56"/>
-      <c r="JE4" s="56"/>
-      <c r="JF4" s="56"/>
-      <c r="JG4" s="56" t="s">
+      <c r="IX4" s="74"/>
+      <c r="IY4" s="74"/>
+      <c r="IZ4" s="74"/>
+      <c r="JA4" s="74"/>
+      <c r="JB4" s="74"/>
+      <c r="JC4" s="74"/>
+      <c r="JD4" s="74"/>
+      <c r="JE4" s="74"/>
+      <c r="JF4" s="74"/>
+      <c r="JG4" s="74" t="s">
         <v>30</v>
       </c>
-      <c r="JH4" s="56"/>
-      <c r="JI4" s="56"/>
-      <c r="JJ4" s="56"/>
-      <c r="JK4" s="56"/>
-      <c r="JL4" s="56"/>
-      <c r="JM4" s="56"/>
-      <c r="JN4" s="56"/>
-      <c r="JO4" s="56"/>
-      <c r="JP4" s="56"/>
-      <c r="JQ4" s="56" t="s">
+      <c r="JH4" s="74"/>
+      <c r="JI4" s="74"/>
+      <c r="JJ4" s="74"/>
+      <c r="JK4" s="74"/>
+      <c r="JL4" s="74"/>
+      <c r="JM4" s="74"/>
+      <c r="JN4" s="74"/>
+      <c r="JO4" s="74"/>
+      <c r="JP4" s="74"/>
+      <c r="JQ4" s="74" t="s">
         <v>31</v>
       </c>
-      <c r="JR4" s="56"/>
-      <c r="JS4" s="56"/>
-      <c r="JT4" s="56"/>
-      <c r="JU4" s="56"/>
-      <c r="JV4" s="56"/>
-      <c r="JW4" s="56"/>
-      <c r="JX4" s="56"/>
-      <c r="JY4" s="56"/>
-      <c r="JZ4" s="56"/>
-      <c r="KA4" s="56" t="s">
+      <c r="JR4" s="74"/>
+      <c r="JS4" s="74"/>
+      <c r="JT4" s="74"/>
+      <c r="JU4" s="74"/>
+      <c r="JV4" s="74"/>
+      <c r="JW4" s="74"/>
+      <c r="JX4" s="74"/>
+      <c r="JY4" s="74"/>
+      <c r="JZ4" s="74"/>
+      <c r="KA4" s="74" t="s">
         <v>32</v>
       </c>
-      <c r="KB4" s="56"/>
-      <c r="KC4" s="56"/>
-      <c r="KD4" s="56"/>
-      <c r="KE4" s="56"/>
-      <c r="KF4" s="56"/>
-      <c r="KG4" s="56"/>
-      <c r="KH4" s="56"/>
-      <c r="KI4" s="56"/>
-      <c r="KJ4" s="56"/>
-      <c r="KK4" s="56" t="s">
+      <c r="KB4" s="74"/>
+      <c r="KC4" s="74"/>
+      <c r="KD4" s="74"/>
+      <c r="KE4" s="74"/>
+      <c r="KF4" s="74"/>
+      <c r="KG4" s="74"/>
+      <c r="KH4" s="74"/>
+      <c r="KI4" s="74"/>
+      <c r="KJ4" s="74"/>
+      <c r="KK4" s="74" t="s">
         <v>33</v>
       </c>
-      <c r="KL4" s="56"/>
-      <c r="KM4" s="56"/>
-      <c r="KN4" s="56"/>
-      <c r="KO4" s="56"/>
-      <c r="KP4" s="56"/>
-      <c r="KQ4" s="56"/>
-      <c r="KR4" s="56"/>
-      <c r="KS4" s="56"/>
-      <c r="KT4" s="56"/>
-      <c r="KU4" s="57" t="s">
+      <c r="KL4" s="74"/>
+      <c r="KM4" s="74"/>
+      <c r="KN4" s="74"/>
+      <c r="KO4" s="74"/>
+      <c r="KP4" s="74"/>
+      <c r="KQ4" s="74"/>
+      <c r="KR4" s="74"/>
+      <c r="KS4" s="74"/>
+      <c r="KT4" s="74"/>
+      <c r="KU4" s="85" t="s">
         <v>34</v>
       </c>
-      <c r="KV4" s="57"/>
-      <c r="KW4" s="57"/>
-      <c r="KX4" s="57"/>
-      <c r="KY4" s="57"/>
-      <c r="KZ4" s="57"/>
-      <c r="LA4" s="57"/>
-      <c r="LB4" s="57"/>
-      <c r="LC4" s="57"/>
-      <c r="LD4" s="57"/>
-      <c r="LE4" s="57" t="s">
+      <c r="KV4" s="85"/>
+      <c r="KW4" s="85"/>
+      <c r="KX4" s="85"/>
+      <c r="KY4" s="85"/>
+      <c r="KZ4" s="85"/>
+      <c r="LA4" s="85"/>
+      <c r="LB4" s="85"/>
+      <c r="LC4" s="85"/>
+      <c r="LD4" s="85"/>
+      <c r="LE4" s="85" t="s">
         <v>35</v>
       </c>
-      <c r="LF4" s="57"/>
-      <c r="LG4" s="57"/>
-      <c r="LH4" s="57"/>
-      <c r="LI4" s="57"/>
-      <c r="LJ4" s="57"/>
-      <c r="LK4" s="57"/>
-      <c r="LL4" s="57"/>
-      <c r="LM4" s="57"/>
-      <c r="LN4" s="57"/>
-      <c r="LO4" s="57" t="s">
+      <c r="LF4" s="85"/>
+      <c r="LG4" s="85"/>
+      <c r="LH4" s="85"/>
+      <c r="LI4" s="85"/>
+      <c r="LJ4" s="85"/>
+      <c r="LK4" s="85"/>
+      <c r="LL4" s="85"/>
+      <c r="LM4" s="85"/>
+      <c r="LN4" s="85"/>
+      <c r="LO4" s="85" t="s">
         <v>36</v>
       </c>
-      <c r="LP4" s="57"/>
-      <c r="LQ4" s="57"/>
-      <c r="LR4" s="57"/>
-      <c r="LS4" s="57"/>
-      <c r="LT4" s="57"/>
-      <c r="LU4" s="57"/>
-      <c r="LV4" s="57"/>
-      <c r="LW4" s="57"/>
-      <c r="LX4" s="57"/>
-      <c r="LY4" s="57" t="s">
+      <c r="LP4" s="85"/>
+      <c r="LQ4" s="85"/>
+      <c r="LR4" s="85"/>
+      <c r="LS4" s="85"/>
+      <c r="LT4" s="85"/>
+      <c r="LU4" s="85"/>
+      <c r="LV4" s="85"/>
+      <c r="LW4" s="85"/>
+      <c r="LX4" s="85"/>
+      <c r="LY4" s="85" t="s">
         <v>37</v>
       </c>
-      <c r="LZ4" s="57"/>
-      <c r="MA4" s="57"/>
-      <c r="MB4" s="57"/>
-      <c r="MC4" s="57"/>
-      <c r="MD4" s="57"/>
-      <c r="ME4" s="57"/>
-      <c r="MF4" s="57"/>
-      <c r="MG4" s="57"/>
-      <c r="MH4" s="57"/>
-      <c r="MI4" s="54" t="s">
+      <c r="LZ4" s="85"/>
+      <c r="MA4" s="85"/>
+      <c r="MB4" s="85"/>
+      <c r="MC4" s="85"/>
+      <c r="MD4" s="85"/>
+      <c r="ME4" s="85"/>
+      <c r="MF4" s="85"/>
+      <c r="MG4" s="85"/>
+      <c r="MH4" s="85"/>
+      <c r="MI4" s="83" t="s">
         <v>38</v>
       </c>
-      <c r="MJ4" s="54"/>
-      <c r="MK4" s="54"/>
-      <c r="ML4" s="54"/>
-      <c r="MM4" s="54"/>
-      <c r="MN4" s="54"/>
-      <c r="MO4" s="54"/>
-      <c r="MP4" s="54"/>
-      <c r="MQ4" s="54"/>
-      <c r="MR4" s="54"/>
-      <c r="MS4" s="54"/>
-      <c r="MT4" s="54"/>
-      <c r="MU4" s="54"/>
-      <c r="MV4" s="54"/>
-      <c r="MW4" s="55" t="s">
+      <c r="MJ4" s="83"/>
+      <c r="MK4" s="83"/>
+      <c r="ML4" s="83"/>
+      <c r="MM4" s="83"/>
+      <c r="MN4" s="83"/>
+      <c r="MO4" s="83"/>
+      <c r="MP4" s="83"/>
+      <c r="MQ4" s="83"/>
+      <c r="MR4" s="83"/>
+      <c r="MS4" s="83"/>
+      <c r="MT4" s="83"/>
+      <c r="MU4" s="83"/>
+      <c r="MV4" s="83"/>
+      <c r="MW4" s="84" t="s">
         <v>39</v>
       </c>
-      <c r="MX4" s="55"/>
-      <c r="MY4" s="55"/>
+      <c r="MX4" s="84"/>
+      <c r="MY4" s="84"/>
       <c r="MZ4" s="26"/>
-      <c r="NA4" s="55" t="s">
+      <c r="NA4" s="84" t="s">
         <v>40</v>
       </c>
-      <c r="NB4" s="55"/>
-      <c r="NC4" s="55"/>
-      <c r="ND4" s="55"/>
-      <c r="NE4" s="55"/>
-      <c r="NF4" s="55"/>
-      <c r="NG4" s="80" t="s">
+      <c r="NB4" s="84"/>
+      <c r="NC4" s="84"/>
+      <c r="ND4" s="84"/>
+      <c r="NE4" s="84"/>
+      <c r="NF4" s="84"/>
+      <c r="NG4" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="NH4" s="84"/>
-      <c r="NI4" s="81"/>
+      <c r="NH4" s="57"/>
+      <c r="NI4" s="58"/>
       <c r="NJ4" s="27"/>
     </row>
     <row r="5" spans="1:374" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="75"/>
-      <c r="B5" s="75"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="76"/>
-      <c r="E5" s="76"/>
-      <c r="F5" s="76"/>
-      <c r="G5" s="76"/>
-      <c r="H5" s="76"/>
-      <c r="I5" s="77"/>
-      <c r="J5" s="77"/>
-      <c r="K5" s="77"/>
-      <c r="L5" s="77"/>
-      <c r="M5" s="77"/>
-      <c r="N5" s="68"/>
-      <c r="O5" s="68"/>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="69"/>
-      <c r="R5" s="69"/>
-      <c r="S5" s="69"/>
-      <c r="T5" s="69"/>
-      <c r="U5" s="69"/>
-      <c r="V5" s="70"/>
-      <c r="W5" s="70"/>
-      <c r="X5" s="70"/>
-      <c r="Y5" s="70"/>
-      <c r="Z5" s="70"/>
-      <c r="AA5" s="70"/>
-      <c r="AB5" s="70"/>
-      <c r="AC5" s="71"/>
-      <c r="AD5" s="71"/>
-      <c r="AE5" s="71"/>
-      <c r="AF5" s="72"/>
-      <c r="AG5" s="72"/>
-      <c r="AH5" s="66"/>
-      <c r="AI5" s="66"/>
-      <c r="AJ5" s="66"/>
-      <c r="AK5" s="66"/>
-      <c r="AL5" s="66"/>
-      <c r="AM5" s="67"/>
-      <c r="AN5" s="67"/>
-      <c r="AO5" s="67"/>
-      <c r="AP5" s="67"/>
-      <c r="AQ5" s="67"/>
-      <c r="AR5" s="67"/>
-      <c r="AS5" s="67"/>
-      <c r="AT5" s="67"/>
-      <c r="AU5" s="67"/>
-      <c r="AV5" s="67"/>
-      <c r="AW5" s="67"/>
-      <c r="AX5" s="67"/>
-      <c r="AY5" s="67"/>
-      <c r="AZ5" s="67"/>
-      <c r="BA5" s="67"/>
-      <c r="BB5" s="67"/>
-      <c r="BC5" s="67"/>
-      <c r="BD5" s="67"/>
-      <c r="BE5" s="67"/>
-      <c r="BF5" s="67"/>
-      <c r="BG5" s="67"/>
-      <c r="BH5" s="67"/>
-      <c r="BI5" s="67"/>
-      <c r="BJ5" s="67"/>
-      <c r="BK5" s="67"/>
-      <c r="BL5" s="67"/>
-      <c r="BM5" s="67"/>
-      <c r="BN5" s="67"/>
+      <c r="A5" s="64"/>
+      <c r="B5" s="64"/>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="66"/>
+      <c r="J5" s="66"/>
+      <c r="K5" s="66"/>
+      <c r="L5" s="66"/>
+      <c r="M5" s="66"/>
+      <c r="N5" s="67"/>
+      <c r="O5" s="67"/>
+      <c r="P5" s="67"/>
+      <c r="Q5" s="68"/>
+      <c r="R5" s="68"/>
+      <c r="S5" s="68"/>
+      <c r="T5" s="68"/>
+      <c r="U5" s="68"/>
+      <c r="V5" s="69"/>
+      <c r="W5" s="69"/>
+      <c r="X5" s="69"/>
+      <c r="Y5" s="69"/>
+      <c r="Z5" s="69"/>
+      <c r="AA5" s="69"/>
+      <c r="AB5" s="69"/>
+      <c r="AC5" s="70"/>
+      <c r="AD5" s="70"/>
+      <c r="AE5" s="70"/>
+      <c r="AF5" s="71"/>
+      <c r="AG5" s="71"/>
+      <c r="AH5" s="72"/>
+      <c r="AI5" s="72"/>
+      <c r="AJ5" s="72"/>
+      <c r="AK5" s="72"/>
+      <c r="AL5" s="72"/>
+      <c r="AM5" s="73"/>
+      <c r="AN5" s="73"/>
+      <c r="AO5" s="73"/>
+      <c r="AP5" s="73"/>
+      <c r="AQ5" s="73"/>
+      <c r="AR5" s="73"/>
+      <c r="AS5" s="73"/>
+      <c r="AT5" s="73"/>
+      <c r="AU5" s="73"/>
+      <c r="AV5" s="73"/>
+      <c r="AW5" s="73"/>
+      <c r="AX5" s="73"/>
+      <c r="AY5" s="73"/>
+      <c r="AZ5" s="73"/>
+      <c r="BA5" s="73"/>
+      <c r="BB5" s="73"/>
+      <c r="BC5" s="73"/>
+      <c r="BD5" s="73"/>
+      <c r="BE5" s="73"/>
+      <c r="BF5" s="73"/>
+      <c r="BG5" s="73"/>
+      <c r="BH5" s="73"/>
+      <c r="BI5" s="73"/>
+      <c r="BJ5" s="73"/>
+      <c r="BK5" s="73"/>
+      <c r="BL5" s="73"/>
+      <c r="BM5" s="73"/>
+      <c r="BN5" s="73"/>
       <c r="BO5" s="28" t="s">
         <v>42</v>
       </c>
@@ -4765,33 +4765,33 @@
       <c r="MH5" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="MI5" s="54"/>
-      <c r="MJ5" s="54"/>
-      <c r="MK5" s="54"/>
-      <c r="ML5" s="54"/>
-      <c r="MM5" s="54"/>
-      <c r="MN5" s="54"/>
-      <c r="MO5" s="54"/>
-      <c r="MP5" s="54"/>
-      <c r="MQ5" s="54"/>
-      <c r="MR5" s="54"/>
-      <c r="MS5" s="54"/>
-      <c r="MT5" s="54"/>
-      <c r="MU5" s="54"/>
-      <c r="MV5" s="54"/>
-      <c r="MW5" s="55"/>
-      <c r="MX5" s="55"/>
-      <c r="MY5" s="55"/>
+      <c r="MI5" s="83"/>
+      <c r="MJ5" s="83"/>
+      <c r="MK5" s="83"/>
+      <c r="ML5" s="83"/>
+      <c r="MM5" s="83"/>
+      <c r="MN5" s="83"/>
+      <c r="MO5" s="83"/>
+      <c r="MP5" s="83"/>
+      <c r="MQ5" s="83"/>
+      <c r="MR5" s="83"/>
+      <c r="MS5" s="83"/>
+      <c r="MT5" s="83"/>
+      <c r="MU5" s="83"/>
+      <c r="MV5" s="83"/>
+      <c r="MW5" s="84"/>
+      <c r="MX5" s="84"/>
+      <c r="MY5" s="84"/>
       <c r="MZ5" s="26"/>
-      <c r="NA5" s="55"/>
-      <c r="NB5" s="55"/>
-      <c r="NC5" s="55"/>
-      <c r="ND5" s="55"/>
-      <c r="NE5" s="55"/>
-      <c r="NF5" s="55"/>
-      <c r="NG5" s="82"/>
-      <c r="NH5" s="85"/>
-      <c r="NI5" s="83"/>
+      <c r="NA5" s="84"/>
+      <c r="NB5" s="84"/>
+      <c r="NC5" s="84"/>
+      <c r="ND5" s="84"/>
+      <c r="NE5" s="84"/>
+      <c r="NF5" s="84"/>
+      <c r="NG5" s="59"/>
+      <c r="NH5" s="60"/>
+      <c r="NI5" s="61"/>
       <c r="NJ5" s="30"/>
     </row>
     <row r="6" spans="1:374" ht="81.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -5908,10 +5908,10 @@
       <c r="NG6" s="40" t="s">
         <v>418</v>
       </c>
-      <c r="NH6" s="78" t="s">
+      <c r="NH6" s="54" t="s">
         <v>419</v>
       </c>
-      <c r="NI6" s="79"/>
+      <c r="NI6" s="55"/>
       <c r="NJ6" s="40" t="s">
         <v>420</v>
       </c>
@@ -6068,43 +6068,43 @@
         <v>0</v>
       </c>
       <c r="BO7" s="52">
-        <f>BY7+CI7+CS7+DC7+DM7+DW7+EG7+EQ7+FA7+FK7+FU7+GE7+GO7+GY7</f>
+        <f t="shared" ref="BO7:BX7" si="0">BY7+CI7+CS7+DC7+DM7+DW7+EG7+EQ7+FA7+FK7+FU7+GE7+GO7+GY7</f>
         <v>0</v>
       </c>
       <c r="BP7" s="52">
-        <f>BZ7+CJ7+CT7+DD7+DN7+DX7+EH7+ER7+FB7+FL7+FV7+GF7+GP7+GZ7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BQ7" s="52">
-        <f>CA7+CK7+CU7+DE7+DO7+DY7+EI7+ES7+FC7+FM7+FW7+GG7+GQ7+HA7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BR7" s="52">
-        <f>CB7+CL7+CV7+DF7+DP7+DZ7+EJ7+ET7+FD7+FN7+FX7+GH7+GR7+HB7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BS7" s="52">
-        <f>CC7+CM7+CW7+DG7+DQ7+EA7+EK7+EU7+FE7+FO7+FY7+GI7+GS7+HC7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BT7" s="52">
-        <f>CD7+CN7+CX7+DH7+DR7+EB7+EL7+EV7+FF7+FP7+FZ7+GJ7+GT7+HD7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BU7" s="52">
-        <f>CE7+CO7+CY7+DI7+DS7+EC7+EM7+EW7+FG7+FQ7+GA7+GK7+GU7+HE7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BV7" s="52">
-        <f>CF7+CP7+CZ7+DJ7+DT7+ED7+EN7+EX7+FH7+FR7+GB7+GL7+GV7+HF7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BW7" s="52">
-        <f>CG7+CQ7+DA7+DK7+DU7+EE7+EO7+EY7+FI7+FS7+GC7+GM7+GW7+HG7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BX7" s="52">
-        <f>CH7+CR7+DB7+DL7+DV7+EF7+EP7+EZ7+FJ7+FT7+GD7+GN7+GX7+HH7</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="BY7" s="47"/>
@@ -6409,6 +6409,35 @@
   </sheetData>
   <autoFilter ref="A6:MZ6" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="45">
+    <mergeCell ref="KA4:KJ4"/>
+    <mergeCell ref="MI4:MV5"/>
+    <mergeCell ref="MW4:MY5"/>
+    <mergeCell ref="NA4:NF5"/>
+    <mergeCell ref="KK4:KT4"/>
+    <mergeCell ref="KU4:LD4"/>
+    <mergeCell ref="LE4:LN4"/>
+    <mergeCell ref="LO4:LX4"/>
+    <mergeCell ref="LY4:MH4"/>
+    <mergeCell ref="IC4:IL4"/>
+    <mergeCell ref="IM4:IV4"/>
+    <mergeCell ref="IW4:JF4"/>
+    <mergeCell ref="JG4:JP4"/>
+    <mergeCell ref="JQ4:JZ4"/>
+    <mergeCell ref="GE4:GN4"/>
+    <mergeCell ref="GO4:GX4"/>
+    <mergeCell ref="GY4:HH4"/>
+    <mergeCell ref="HI4:HR4"/>
+    <mergeCell ref="HS4:IB4"/>
+    <mergeCell ref="EG4:EP4"/>
+    <mergeCell ref="EQ4:EZ4"/>
+    <mergeCell ref="FA4:FJ4"/>
+    <mergeCell ref="FK4:FT4"/>
+    <mergeCell ref="FU4:GD4"/>
+    <mergeCell ref="CI4:CR4"/>
+    <mergeCell ref="CS4:DB4"/>
+    <mergeCell ref="DC4:DL4"/>
+    <mergeCell ref="DM4:DV4"/>
+    <mergeCell ref="DW4:EF4"/>
     <mergeCell ref="NH6:NI6"/>
     <mergeCell ref="NG4:NI5"/>
     <mergeCell ref="A1:B1"/>
@@ -6425,35 +6454,6 @@
     <mergeCell ref="AM4:BN5"/>
     <mergeCell ref="BO4:BX4"/>
     <mergeCell ref="BY4:CH4"/>
-    <mergeCell ref="CI4:CR4"/>
-    <mergeCell ref="CS4:DB4"/>
-    <mergeCell ref="DC4:DL4"/>
-    <mergeCell ref="DM4:DV4"/>
-    <mergeCell ref="DW4:EF4"/>
-    <mergeCell ref="EG4:EP4"/>
-    <mergeCell ref="EQ4:EZ4"/>
-    <mergeCell ref="FA4:FJ4"/>
-    <mergeCell ref="FK4:FT4"/>
-    <mergeCell ref="FU4:GD4"/>
-    <mergeCell ref="GE4:GN4"/>
-    <mergeCell ref="GO4:GX4"/>
-    <mergeCell ref="GY4:HH4"/>
-    <mergeCell ref="HI4:HR4"/>
-    <mergeCell ref="HS4:IB4"/>
-    <mergeCell ref="IC4:IL4"/>
-    <mergeCell ref="IM4:IV4"/>
-    <mergeCell ref="IW4:JF4"/>
-    <mergeCell ref="JG4:JP4"/>
-    <mergeCell ref="JQ4:JZ4"/>
-    <mergeCell ref="KA4:KJ4"/>
-    <mergeCell ref="MI4:MV5"/>
-    <mergeCell ref="MW4:MY5"/>
-    <mergeCell ref="NA4:NF5"/>
-    <mergeCell ref="KK4:KT4"/>
-    <mergeCell ref="KU4:LD4"/>
-    <mergeCell ref="LE4:LN4"/>
-    <mergeCell ref="LO4:LX4"/>
-    <mergeCell ref="LY4:MH4"/>
   </mergeCells>
   <conditionalFormatting sqref="A1:A6">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>

</xml_diff>